<commit_message>
Add ContAgil monthly SELIC/TJLP loaders to Polars summary.
Supports ContAgil Bacen Selic (% a.d.) and tjlp_mensal.xlsx via --tjlp,
joins TJLP into taxa_contrato_efetiva, and capitalizes impact with
cumprod factors instead of a flat product of all rates.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_fluxos_polars.xlsx
+++ b/output/resumo_fluxos_polars.xlsx
@@ -726,7 +726,9 @@
       <c r="E9" s="3">
         <v>4166.67</v>
       </c>
-      <c r="F9" s="3"/>
+      <c r="F9" s="3">
+        <v>3.744151755248671</v>
+      </c>
       <c r="G9" s="1">
         <v>117</v>
       </c>
@@ -747,7 +749,9 @@
       <c r="E10" s="3">
         <v>4375</v>
       </c>
-      <c r="F10" s="3"/>
+      <c r="F10" s="3">
+        <v>6.221197630385841</v>
+      </c>
       <c r="G10" s="1">
         <v>162</v>
       </c>
@@ -883,7 +887,9 @@
       <c r="E16" s="3">
         <v>1666.67</v>
       </c>
-      <c r="F16" s="3"/>
+      <c r="F16" s="3">
+        <v>3.382589776576153</v>
+      </c>
       <c r="G16" s="1">
         <v>108</v>
       </c>
@@ -927,7 +933,9 @@
       <c r="E18" s="3">
         <v>2444.44</v>
       </c>
-      <c r="F18" s="3"/>
+      <c r="F18" s="3">
+        <v>3.744151755248671</v>
+      </c>
       <c r="G18" s="1">
         <v>117</v>
       </c>

</xml_diff>

<commit_message>
Use ContAgil monthly SELIC/TJLP only (no daily series).
Defaults --selic/--tjlp to selic_mensal.xlsx and tjlp_mensal.xlsx,
capitalizes both series monthly via cumprod, and drops STP/daily SELIC.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_fluxos_polars.xlsx
+++ b/output/resumo_fluxos_polars.xlsx
@@ -560,13 +560,13 @@
         <v>59292.6</v>
       </c>
       <c r="D2" s="3">
-        <v>262490.73</v>
+        <v>324805.17</v>
       </c>
       <c r="E2" s="3">
         <v>2083.33</v>
       </c>
       <c r="F2" s="3">
-        <v>2.847338410355227</v>
+        <v>1.950483811861024</v>
       </c>
       <c r="G2" s="1">
         <v>162</v>
@@ -583,13 +583,13 @@
         <v>172757.55</v>
       </c>
       <c r="D3" s="3">
-        <v>743647.38</v>
+        <v>916557.6</v>
       </c>
       <c r="E3" s="3">
         <v>4166.67</v>
       </c>
       <c r="F3" s="3">
-        <v>3.651366415824136</v>
+        <v>2.348828657415724</v>
       </c>
       <c r="G3" s="1">
         <v>189</v>
@@ -606,13 +606,13 @@
         <v>15799.41</v>
       </c>
       <c r="D4" s="3">
-        <v>71659.89</v>
+        <v>88779.12</v>
       </c>
       <c r="E4" s="3">
         <v>1388.89</v>
       </c>
       <c r="F4" s="3">
-        <v>1.846239621373051</v>
+        <v>1.434402850537668</v>
       </c>
       <c r="G4" s="1">
         <v>108</v>
@@ -629,13 +629,13 @@
         <v>76582.14999999999</v>
       </c>
       <c r="D5" s="3">
-        <v>305408.73</v>
+        <v>372302.64</v>
       </c>
       <c r="E5" s="3">
         <v>2500</v>
       </c>
       <c r="F5" s="3">
-        <v>2.123305046609123</v>
+        <v>1.176386332273652</v>
       </c>
       <c r="G5" s="1">
         <v>252</v>
@@ -652,13 +652,13 @@
         <v>50117.52</v>
       </c>
       <c r="D6" s="3">
-        <v>213435.6</v>
+        <v>262516.05</v>
       </c>
       <c r="E6" s="3">
         <v>1875</v>
       </c>
       <c r="F6" s="3">
-        <v>2.672281641848591</v>
+        <v>1.830294826634917</v>
       </c>
       <c r="G6" s="1">
         <v>162</v>
@@ -675,13 +675,13 @@
         <v>88910.2</v>
       </c>
       <c r="D7" s="3">
-        <v>365274.67</v>
+        <v>446848.08</v>
       </c>
       <c r="E7" s="3">
         <v>5333.33</v>
       </c>
       <c r="F7" s="3">
-        <v>1.676494741941926</v>
+        <v>1.053949153431416</v>
       </c>
       <c r="G7" s="1">
         <v>198</v>
@@ -698,13 +698,13 @@
         <v>13819.32</v>
       </c>
       <c r="D8" s="3">
-        <v>62748.81</v>
+        <v>77528.52</v>
       </c>
       <c r="E8" s="3">
         <v>3125</v>
       </c>
       <c r="F8" s="3">
-        <v>1.423206117087701</v>
+        <v>1.20263287207859</v>
       </c>
       <c r="G8" s="1">
         <v>72</v>
@@ -721,13 +721,13 @@
         <v>62694.66</v>
       </c>
       <c r="D9" s="3">
-        <v>271072.8</v>
+        <v>333733.35</v>
       </c>
       <c r="E9" s="3">
         <v>4166.67</v>
       </c>
       <c r="F9" s="3">
-        <v>3.744151755248671</v>
+        <v>2.852767969898418</v>
       </c>
       <c r="G9" s="1">
         <v>117</v>
@@ -744,13 +744,13 @@
         <v>132120.78</v>
       </c>
       <c r="D10" s="3">
-        <v>545375.73</v>
+        <v>667686.9</v>
       </c>
       <c r="E10" s="3">
         <v>4375</v>
       </c>
       <c r="F10" s="3">
-        <v>6.221197630385841</v>
+        <v>4.269420493312508</v>
       </c>
       <c r="G10" s="1">
         <v>162</v>
@@ -767,13 +767,13 @@
         <v>7954.05</v>
       </c>
       <c r="D11" s="3">
-        <v>35281.71</v>
+        <v>43440</v>
       </c>
       <c r="E11" s="3">
         <v>1666.67</v>
       </c>
       <c r="F11" s="3">
-        <v>1.463433948770676</v>
+        <v>1.236706760153628</v>
       </c>
       <c r="G11" s="1">
         <v>72</v>
@@ -790,13 +790,13 @@
         <v>270792.98</v>
       </c>
       <c r="D12" s="3">
-        <v>992544.6899999999</v>
+        <v>1198974.74</v>
       </c>
       <c r="E12" s="3">
         <v>5952.38</v>
       </c>
       <c r="F12" s="3">
-        <v>2.637752274653645</v>
+        <v>1.343524304820472</v>
       </c>
       <c r="G12" s="1">
         <v>288</v>
@@ -813,13 +813,13 @@
         <v>85148.13</v>
       </c>
       <c r="D13" s="3">
-        <v>333741.06</v>
+        <v>405542.73</v>
       </c>
       <c r="E13" s="3">
         <v>2000</v>
       </c>
       <c r="F13" s="3">
-        <v>3.592738024733769</v>
+        <v>2.262655460611077</v>
       </c>
       <c r="G13" s="1">
         <v>198</v>
@@ -836,13 +836,13 @@
         <v>53890.02</v>
       </c>
       <c r="D14" s="3">
-        <v>217319.76</v>
+        <v>265315.65</v>
       </c>
       <c r="E14" s="3">
         <v>1979.17</v>
       </c>
       <c r="F14" s="3">
-        <v>2.85312665832283</v>
+        <v>1.996241073224543</v>
       </c>
       <c r="G14" s="1">
         <v>153</v>
@@ -859,13 +859,13 @@
         <v>255027</v>
       </c>
       <c r="D15" s="3">
-        <v>955945.65</v>
+        <v>1155614.19</v>
       </c>
       <c r="E15" s="3">
         <v>3819.44</v>
       </c>
       <c r="F15" s="3">
-        <v>5.451218198869583</v>
+        <v>3.157644335379528</v>
       </c>
       <c r="G15" s="1">
         <v>234</v>
@@ -882,13 +882,13 @@
         <v>18959.28</v>
       </c>
       <c r="D16" s="3">
-        <v>78068.31</v>
+        <v>95674.92</v>
       </c>
       <c r="E16" s="3">
         <v>1666.67</v>
       </c>
       <c r="F16" s="3">
-        <v>3.382589776576153</v>
+        <v>2.631758010979339</v>
       </c>
       <c r="G16" s="1">
         <v>108</v>
@@ -905,13 +905,13 @@
         <v>126759.89</v>
       </c>
       <c r="D17" s="3">
-        <v>468780.57</v>
+        <v>565859.9300000001</v>
       </c>
       <c r="E17" s="3">
         <v>5666.67</v>
       </c>
       <c r="F17" s="3">
-        <v>1.90676133142373</v>
+        <v>1.149400556072266</v>
       </c>
       <c r="G17" s="1">
         <v>216</v>
@@ -928,13 +928,13 @@
         <v>34543.62</v>
       </c>
       <c r="D18" s="3">
-        <v>137583.27</v>
+        <v>168122.28</v>
       </c>
       <c r="E18" s="3">
         <v>2444.44</v>
       </c>
       <c r="F18" s="3">
-        <v>3.744151755248671</v>
+        <v>2.852767969898418</v>
       </c>
       <c r="G18" s="1">
         <v>117</v>
@@ -951,13 +951,13 @@
         <v>97517.75999999999</v>
       </c>
       <c r="D19" s="3">
-        <v>371541.12</v>
+        <v>450581.97</v>
       </c>
       <c r="E19" s="3">
         <v>3229.17</v>
       </c>
       <c r="F19" s="3">
-        <v>3.034622285954255</v>
+        <v>2.079086577095331</v>
       </c>
       <c r="G19" s="1">
         <v>162</v>
@@ -974,13 +974,13 @@
         <v>175218.57</v>
       </c>
       <c r="D20" s="3">
-        <v>643926.36</v>
+        <v>776805.1800000001</v>
       </c>
       <c r="E20" s="3">
         <v>3666.67</v>
       </c>
       <c r="F20" s="3">
-        <v>4.199396323087085</v>
+        <v>2.645684797388774</v>
       </c>
       <c r="G20" s="1">
         <v>198</v>
@@ -997,13 +997,13 @@
         <v>52391.34</v>
       </c>
       <c r="D21" s="3">
-        <v>199574.67</v>
+        <v>242262.36</v>
       </c>
       <c r="E21" s="3">
         <v>2291.67</v>
       </c>
       <c r="F21" s="3">
-        <v>2.534812586278763</v>
+        <v>1.810941041535916</v>
       </c>
       <c r="G21" s="1">
         <v>144</v>
@@ -1053,7 +1053,7 @@
         <v>17690.01</v>
       </c>
       <c r="D2" s="3">
-        <v>85081.89</v>
+        <v>106425.98</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1067,7 +1067,7 @@
         <v>9010.530000000001</v>
       </c>
       <c r="D3" s="3">
-        <v>42865.74</v>
+        <v>53441.79</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1081,7 +1081,7 @@
         <v>68652.33</v>
       </c>
       <c r="D4" s="3">
-        <v>334351.71</v>
+        <v>419387.07</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1095,7 +1095,7 @@
         <v>5479.98</v>
       </c>
       <c r="D5" s="3">
-        <v>26518.59</v>
+        <v>33223.44</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1109,7 +1109,7 @@
         <v>9743.6</v>
       </c>
       <c r="D6" s="3">
-        <v>46612.54</v>
+        <v>58214.22</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1123,7 +1123,7 @@
         <v>51367.67</v>
       </c>
       <c r="D7" s="3">
-        <v>230346.91</v>
+        <v>283504.48</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1137,7 +1137,7 @@
         <v>6575.94</v>
       </c>
       <c r="D8" s="3">
-        <v>29151.99</v>
+        <v>35803.86</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1151,7 +1151,7 @@
         <v>39105.36</v>
       </c>
       <c r="D9" s="3">
-        <v>177245.28</v>
+        <v>218454.78</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1165,7 +1165,7 @@
         <v>145436.61</v>
       </c>
       <c r="D10" s="3">
-        <v>655388.88</v>
+        <v>807095.1</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1179,7 +1179,7 @@
         <v>25233.45</v>
       </c>
       <c r="D11" s="3">
-        <v>112791.12</v>
+        <v>138693.48</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1193,7 +1193,7 @@
         <v>64256.5</v>
       </c>
       <c r="D12" s="3">
-        <v>287569.6</v>
+        <v>353759.17</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1207,7 +1207,7 @@
         <v>19002.54</v>
       </c>
       <c r="D13" s="3">
-        <v>85152.03</v>
+        <v>104809.47</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -1221,7 +1221,7 @@
         <v>75325.53</v>
       </c>
       <c r="D14" s="3">
-        <v>337074.52</v>
+        <v>414557.31</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1235,7 +1235,7 @@
         <v>64155.9</v>
       </c>
       <c r="D15" s="3">
-        <v>261596.65</v>
+        <v>321018.2</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1249,7 +1249,7 @@
         <v>8027.79</v>
       </c>
       <c r="D16" s="3">
-        <v>32839.26</v>
+        <v>40293.66</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1263,7 +1263,7 @@
         <v>21027.09</v>
       </c>
       <c r="D17" s="3">
-        <v>86273.52</v>
+        <v>105845.13</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -1277,7 +1277,7 @@
         <v>142821.12</v>
       </c>
       <c r="D18" s="3">
-        <v>583174.77</v>
+        <v>715602.9300000001</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -1291,7 +1291,7 @@
         <v>45747.9</v>
       </c>
       <c r="D19" s="3">
-        <v>186713.1</v>
+        <v>229116.63</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -1305,7 +1305,7 @@
         <v>111736.71</v>
       </c>
       <c r="D20" s="3">
-        <v>455536.86</v>
+        <v>559013.67</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -1319,7 +1319,7 @@
         <v>21140.82</v>
       </c>
       <c r="D21" s="3">
-        <v>86588.52</v>
+        <v>106238.88</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -1333,7 +1333,7 @@
         <v>86186.3</v>
       </c>
       <c r="D22" s="3">
-        <v>351575.84</v>
+        <v>431429.2</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -1347,7 +1347,7 @@
         <v>50301.92</v>
       </c>
       <c r="D23" s="3">
-        <v>185733.64</v>
+        <v>226324.72</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -1361,7 +1361,7 @@
         <v>3928.5</v>
       </c>
       <c r="D24" s="3">
-        <v>14577.21</v>
+        <v>17791.74</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -1375,7 +1375,7 @@
         <v>7290</v>
       </c>
       <c r="D25" s="3">
-        <v>27150.45</v>
+        <v>33177.42</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -1389,7 +1389,7 @@
         <v>96545.64</v>
       </c>
       <c r="D26" s="3">
-        <v>356912.1</v>
+        <v>435085.35</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -1403,7 +1403,7 @@
         <v>33733.68</v>
       </c>
       <c r="D27" s="3">
-        <v>124601.7</v>
+        <v>151850.31</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1417,7 +1417,7 @@
         <v>92557.09</v>
       </c>
       <c r="D28" s="3">
-        <v>341558.17</v>
+        <v>416124.59</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -1431,7 +1431,7 @@
         <v>9728.16</v>
       </c>
       <c r="D29" s="3">
-        <v>36044.01</v>
+        <v>43969.11</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -1445,7 +1445,7 @@
         <v>68338.89999999999</v>
       </c>
       <c r="D30" s="3">
-        <v>252262.49</v>
+        <v>307364.6</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -1459,7 +1459,7 @@
         <v>35056.01</v>
       </c>
       <c r="D31" s="3">
-        <v>120287.29</v>
+        <v>141815.52</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -1473,7 +1473,7 @@
         <v>427.05</v>
       </c>
       <c r="D32" s="3">
-        <v>1499.85</v>
+        <v>1785.66</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -1487,7 +1487,7 @@
         <v>81</v>
       </c>
       <c r="D33" s="3">
-        <v>286.62</v>
+        <v>342.75</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -1501,7 +1501,7 @@
         <v>50113.8</v>
       </c>
       <c r="D34" s="3">
-        <v>172481.25</v>
+        <v>203580.12</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -1515,7 +1515,7 @@
         <v>21719.34</v>
       </c>
       <c r="D35" s="3">
-        <v>74582.49000000001</v>
+        <v>87955.38</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -1529,7 +1529,7 @@
         <v>72517.89</v>
       </c>
       <c r="D36" s="3">
-        <v>248573.96</v>
+        <v>292951.34</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -1543,7 +1543,7 @@
         <v>2945.58</v>
       </c>
       <c r="D37" s="3">
-        <v>10221.72</v>
+        <v>12100.5</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -1557,7 +1557,7 @@
         <v>50491.48</v>
       </c>
       <c r="D38" s="3">
-        <v>173159.41</v>
+        <v>204110.57</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -1571,7 +1571,7 @@
         <v>21693.03</v>
       </c>
       <c r="D39" s="3">
-        <v>67951.63</v>
+        <v>78845.64</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -1585,7 +1585,7 @@
         <v>11609.55</v>
       </c>
       <c r="D40" s="3">
-        <v>36896.85</v>
+        <v>42840.93</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -1599,7 +1599,7 @@
         <v>9705.42</v>
       </c>
       <c r="D41" s="3">
-        <v>30597.15</v>
+        <v>35510.82</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -1613,7 +1613,7 @@
         <v>52479.12</v>
       </c>
       <c r="D42" s="3">
-        <v>164242.93</v>
+        <v>190567.75</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -1627,7 +1627,7 @@
         <v>32644.03</v>
       </c>
       <c r="D43" s="3">
-        <v>102309.39</v>
+        <v>118713.75</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -1641,7 +1641,7 @@
         <v>11342.6</v>
       </c>
       <c r="D44" s="3">
-        <v>31913.88</v>
+        <v>37162.87</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -1655,7 +1655,7 @@
         <v>399.66</v>
       </c>
       <c r="D45" s="3">
-        <v>1169.16</v>
+        <v>1355.79</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -1669,7 +1669,7 @@
         <v>1399.68</v>
       </c>
       <c r="D46" s="3">
-        <v>4030.17</v>
+        <v>4678.47</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -1683,7 +1683,7 @@
         <v>32440.15</v>
       </c>
       <c r="D47" s="3">
-        <v>91000.48</v>
+        <v>106012.99</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -1697,7 +1697,7 @@
         <v>16623.54</v>
       </c>
       <c r="D48" s="3">
-        <v>46700.04</v>
+        <v>54393.64</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -1711,7 +1711,7 @@
         <v>1852.42</v>
       </c>
       <c r="D49" s="3">
-        <v>4713.01</v>
+        <v>5581.21</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -1725,7 +1725,7 @@
         <v>14641.42</v>
       </c>
       <c r="D50" s="3">
-        <v>36154.28</v>
+        <v>43051.32</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -1739,7 +1739,7 @@
         <v>4583.82</v>
       </c>
       <c r="D51" s="3">
-        <v>11526.09</v>
+        <v>13678.98</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -1753,7 +1753,7 @@
         <v>5323.52</v>
       </c>
       <c r="D52" s="3">
-        <v>11711.94</v>
+        <v>14152.89</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -1767,7 +1767,7 @@
         <v>59.15</v>
       </c>
       <c r="D53" s="3">
-        <v>122.83</v>
+        <v>146.2</v>
       </c>
     </row>
   </sheetData>
@@ -1814,7 +1814,7 @@
         <v>515578.71</v>
       </c>
       <c r="D2" s="3">
-        <v>2140374.72</v>
+        <v>2624947.29</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1828,7 +1828,7 @@
         <v>446011.55</v>
       </c>
       <c r="D3" s="3">
-        <v>1636471.05</v>
+        <v>1975779.92</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1842,7 +1842,7 @@
         <v>343937.2</v>
       </c>
       <c r="D4" s="3">
-        <v>1321220.32</v>
+        <v>1602462.27</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1856,7 +1856,7 @@
         <v>253459.56</v>
       </c>
       <c r="D5" s="3">
-        <v>987624.9</v>
+        <v>1200678.62</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1870,7 +1870,7 @@
         <v>137539.47</v>
       </c>
       <c r="D6" s="3">
-        <v>533315.73</v>
+        <v>647805.09</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1884,7 +1884,7 @@
         <v>76513.98</v>
       </c>
       <c r="D7" s="3">
-        <v>333821.61</v>
+        <v>411261.87</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1898,7 +1898,7 @@
         <v>58297.08</v>
       </c>
       <c r="D8" s="3">
-        <v>244524.87</v>
+        <v>300341.4</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1912,7 +1912,7 @@
         <v>18959.28</v>
       </c>
       <c r="D9" s="3">
-        <v>78068.31</v>
+        <v>95674.92</v>
       </c>
     </row>
   </sheetData>
@@ -1956,7 +1956,7 @@
         <v>110576.45</v>
       </c>
       <c r="C2" s="3">
-        <v>535430.47</v>
+        <v>670692.5</v>
       </c>
       <c r="D2" s="1">
         <v>141</v>
@@ -1970,7 +1970,7 @@
         <v>426303.6</v>
       </c>
       <c r="C3" s="3">
-        <v>1914720.33</v>
+        <v>2356677.65</v>
       </c>
       <c r="D3" s="1">
         <v>540</v>
@@ -1984,7 +1984,7 @@
         <v>500843.63</v>
       </c>
       <c r="C4" s="3">
-        <v>2044298.52</v>
+        <v>2508558.3</v>
       </c>
       <c r="D4" s="1">
         <v>711</v>
@@ -1998,7 +1998,7 @@
         <v>362423.89</v>
       </c>
       <c r="C5" s="3">
-        <v>1338839.77</v>
+        <v>1631687.84</v>
       </c>
       <c r="D5" s="1">
         <v>627</v>
@@ -2012,7 +2012,7 @@
         <v>233352.15</v>
       </c>
       <c r="C6" s="3">
-        <v>801092.59</v>
+        <v>944641.84</v>
       </c>
       <c r="D6" s="1">
         <v>543</v>
@@ -2026,7 +2026,7 @@
         <v>128131.15</v>
       </c>
       <c r="C7" s="3">
-        <v>401997.95</v>
+        <v>466478.89</v>
       </c>
       <c r="D7" s="1">
         <v>375</v>
@@ -2040,7 +2040,7 @@
         <v>62205.63</v>
       </c>
       <c r="C8" s="3">
-        <v>174813.73</v>
+        <v>203603.76</v>
       </c>
       <c r="D8" s="1">
         <v>219</v>
@@ -2054,7 +2054,7 @@
         <v>21077.66</v>
       </c>
       <c r="C9" s="3">
-        <v>52393.38</v>
+        <v>62311.51</v>
       </c>
       <c r="D9" s="1">
         <v>117</v>
@@ -2068,7 +2068,7 @@
         <v>5323.52</v>
       </c>
       <c r="C10" s="3">
-        <v>11711.94</v>
+        <v>14152.89</v>
       </c>
       <c r="D10" s="1">
         <v>36</v>
@@ -2082,7 +2082,7 @@
         <v>59.15</v>
       </c>
       <c r="C11" s="3">
-        <v>122.83</v>
+        <v>146.2</v>
       </c>
       <c r="D11" s="1">
         <v>3</v>
@@ -2126,7 +2126,7 @@
         <v>22</v>
       </c>
       <c r="B3" s="3">
-        <v>7275421.51</v>
+        <v>8858951.380000001</v>
       </c>
     </row>
     <row r="4" spans="1:2">

</xml_diff>

<commit_message>
Emit ContAgil executive flow summary report
Regenerate RELATORIO_EXECUTIVO and Polars workbook (indiretas +
OPERACOES DIRETAS sample) and uniquify contrato IDs across files.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/resumo_fluxos_polars.xlsx
+++ b/output/resumo_fluxos_polars.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="27">
   <si>
     <t>contrato</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>BANCO COOPERATIVO DO BRASIL SA - BANCOOB</t>
+  </si>
+  <si>
+    <t>BNDES</t>
   </si>
   <si>
     <t>ano</t>
@@ -164,8 +167,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:G21" totalsRowShown="0">
-  <autoFilter ref="A1:G21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:G24" totalsRowShown="0">
+  <autoFilter ref="A1:G24"/>
   <tableColumns count="7">
     <tableColumn id="1" name="contrato" dataDxfId="0"/>
     <tableColumn id="2" name="Instituição Financeira Credenciada" dataDxfId="1"/>
@@ -180,8 +183,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Frame1" displayName="Frame1" ref="A1:D53" totalsRowShown="0">
-  <autoFilter ref="A1:D53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Frame1" displayName="Frame1" ref="A1:D58" totalsRowShown="0">
+  <autoFilter ref="A1:D58"/>
   <tableColumns count="4">
     <tableColumn id="1" name="ano" dataDxfId="0"/>
     <tableColumn id="2" name="Instituição Financeira Credenciada" dataDxfId="1"/>
@@ -193,8 +196,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Frame2" displayName="Frame2" ref="A1:D9" totalsRowShown="0">
-  <autoFilter ref="A1:D9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Frame2" displayName="Frame2" ref="A1:D10" totalsRowShown="0">
+  <autoFilter ref="A1:D10"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Instituição Financeira Credenciada" dataDxfId="1"/>
     <tableColumn id="2" name="qtd_contratos" dataDxfId="0"/>
@@ -514,7 +517,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -557,19 +560,19 @@
         <v>7</v>
       </c>
       <c r="C2" s="3">
-        <v>59292.6</v>
+        <v>19764.2</v>
       </c>
       <c r="D2" s="3">
-        <v>324805.17</v>
+        <v>108268.39</v>
       </c>
       <c r="E2" s="3">
         <v>2083.33</v>
       </c>
       <c r="F2" s="3">
-        <v>1.950483811861024</v>
+        <v>1.622269401480327</v>
       </c>
       <c r="G2" s="1">
-        <v>162</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -580,19 +583,19 @@
         <v>7</v>
       </c>
       <c r="C3" s="3">
-        <v>172757.55</v>
+        <v>57585.85</v>
       </c>
       <c r="D3" s="3">
-        <v>916557.6</v>
+        <v>305519.2</v>
       </c>
       <c r="E3" s="3">
         <v>4166.67</v>
       </c>
       <c r="F3" s="3">
-        <v>2.348828657415724</v>
+        <v>1.758504455114086</v>
       </c>
       <c r="G3" s="1">
-        <v>189</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -603,19 +606,19 @@
         <v>8</v>
       </c>
       <c r="C4" s="3">
-        <v>15799.41</v>
+        <v>5266.47</v>
       </c>
       <c r="D4" s="3">
-        <v>88779.12</v>
+        <v>29593.04</v>
       </c>
       <c r="E4" s="3">
         <v>1388.89</v>
       </c>
       <c r="F4" s="3">
-        <v>1.434402850537668</v>
+        <v>1.380644873108813</v>
       </c>
       <c r="G4" s="1">
-        <v>108</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -626,19 +629,19 @@
         <v>9</v>
       </c>
       <c r="C5" s="3">
-        <v>76582.14999999999</v>
+        <v>24333.81</v>
       </c>
       <c r="D5" s="3">
-        <v>372302.64</v>
+        <v>118298.38</v>
       </c>
       <c r="E5" s="3">
         <v>2500</v>
       </c>
       <c r="F5" s="3">
-        <v>1.176386332273652</v>
+        <v>2.122550168003448</v>
       </c>
       <c r="G5" s="1">
-        <v>252</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -649,19 +652,19 @@
         <v>9</v>
       </c>
       <c r="C6" s="3">
-        <v>50117.52</v>
+        <v>16705.84</v>
       </c>
       <c r="D6" s="3">
-        <v>262516.05</v>
+        <v>87505.35000000001</v>
       </c>
       <c r="E6" s="3">
         <v>1875</v>
       </c>
       <c r="F6" s="3">
-        <v>1.830294826634917</v>
+        <v>1.622269401480327</v>
       </c>
       <c r="G6" s="1">
-        <v>162</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -672,19 +675,19 @@
         <v>10</v>
       </c>
       <c r="C7" s="3">
-        <v>88910.2</v>
+        <v>27869.86</v>
       </c>
       <c r="D7" s="3">
-        <v>446848.08</v>
+        <v>140069.36</v>
       </c>
       <c r="E7" s="3">
         <v>5333.33</v>
       </c>
       <c r="F7" s="3">
-        <v>1.053949153431416</v>
+        <v>1.806412673934507</v>
       </c>
       <c r="G7" s="1">
-        <v>198</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -695,19 +698,19 @@
         <v>11</v>
       </c>
       <c r="C8" s="3">
-        <v>13819.32</v>
+        <v>4606.44</v>
       </c>
       <c r="D8" s="3">
-        <v>77528.52</v>
+        <v>25842.84</v>
       </c>
       <c r="E8" s="3">
         <v>3125</v>
       </c>
       <c r="F8" s="3">
-        <v>1.20263287207859</v>
+        <v>1.239903796222104</v>
       </c>
       <c r="G8" s="1">
-        <v>72</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -718,19 +721,19 @@
         <v>11</v>
       </c>
       <c r="C9" s="3">
-        <v>62694.66</v>
+        <v>20898.22</v>
       </c>
       <c r="D9" s="3">
-        <v>333733.35</v>
+        <v>111244.45</v>
       </c>
       <c r="E9" s="3">
         <v>4166.67</v>
       </c>
       <c r="F9" s="3">
-        <v>2.852767969898418</v>
+        <v>1.418258787877028</v>
       </c>
       <c r="G9" s="1">
-        <v>117</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -741,19 +744,19 @@
         <v>7</v>
       </c>
       <c r="C10" s="3">
-        <v>132120.78</v>
+        <v>44040.26</v>
       </c>
       <c r="D10" s="3">
-        <v>667686.9</v>
+        <v>222562.3</v>
       </c>
       <c r="E10" s="3">
         <v>4375</v>
       </c>
       <c r="F10" s="3">
-        <v>4.269420493312508</v>
+        <v>1.622269401480327</v>
       </c>
       <c r="G10" s="1">
-        <v>162</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -764,19 +767,19 @@
         <v>8</v>
       </c>
       <c r="C11" s="3">
-        <v>7954.05</v>
+        <v>2651.35</v>
       </c>
       <c r="D11" s="3">
-        <v>43440</v>
+        <v>14480</v>
       </c>
       <c r="E11" s="3">
         <v>1666.67</v>
       </c>
       <c r="F11" s="3">
-        <v>1.236706760153628</v>
+        <v>1.239903796222104</v>
       </c>
       <c r="G11" s="1">
-        <v>72</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -787,19 +790,19 @@
         <v>12</v>
       </c>
       <c r="C12" s="3">
-        <v>270792.98</v>
+        <v>86938.3</v>
       </c>
       <c r="D12" s="3">
-        <v>1198974.74</v>
+        <v>384931.82</v>
       </c>
       <c r="E12" s="3">
         <v>5952.38</v>
       </c>
       <c r="F12" s="3">
-        <v>1.343524304820472</v>
+        <v>2.363480147652739</v>
       </c>
       <c r="G12" s="1">
-        <v>288</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -810,19 +813,19 @@
         <v>13</v>
       </c>
       <c r="C13" s="3">
-        <v>85148.13</v>
+        <v>28382.71</v>
       </c>
       <c r="D13" s="3">
-        <v>405542.73</v>
+        <v>135180.91</v>
       </c>
       <c r="E13" s="3">
         <v>2000</v>
       </c>
       <c r="F13" s="3">
-        <v>2.262655460611077</v>
+        <v>1.806412673934507</v>
       </c>
       <c r="G13" s="1">
-        <v>198</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -833,19 +836,19 @@
         <v>7</v>
       </c>
       <c r="C14" s="3">
-        <v>53890.02</v>
+        <v>17963.34</v>
       </c>
       <c r="D14" s="3">
-        <v>265315.65</v>
+        <v>88438.55</v>
       </c>
       <c r="E14" s="3">
         <v>1979.17</v>
       </c>
       <c r="F14" s="3">
-        <v>1.996241073224543</v>
+        <v>1.579244881893387</v>
       </c>
       <c r="G14" s="1">
-        <v>153</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -856,19 +859,19 @@
         <v>10</v>
       </c>
       <c r="C15" s="3">
-        <v>255027</v>
+        <v>85009</v>
       </c>
       <c r="D15" s="3">
-        <v>1155614.19</v>
+        <v>385204.73</v>
       </c>
       <c r="E15" s="3">
         <v>3819.44</v>
       </c>
       <c r="F15" s="3">
-        <v>3.157644335379528</v>
+        <v>2.011457989390418</v>
       </c>
       <c r="G15" s="1">
-        <v>234</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -879,19 +882,19 @@
         <v>14</v>
       </c>
       <c r="C16" s="3">
-        <v>18959.28</v>
+        <v>6319.76</v>
       </c>
       <c r="D16" s="3">
-        <v>95674.92</v>
+        <v>31891.64</v>
       </c>
       <c r="E16" s="3">
         <v>1666.67</v>
       </c>
       <c r="F16" s="3">
-        <v>2.631758010979339</v>
+        <v>1.380644873108813</v>
       </c>
       <c r="G16" s="1">
-        <v>108</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -902,19 +905,19 @@
         <v>9</v>
       </c>
       <c r="C17" s="3">
-        <v>126759.89</v>
+        <v>40277.61</v>
       </c>
       <c r="D17" s="3">
-        <v>565859.9300000001</v>
+        <v>179800.45</v>
       </c>
       <c r="E17" s="3">
         <v>5666.67</v>
       </c>
       <c r="F17" s="3">
-        <v>1.149400556072266</v>
+        <v>1.90618026564165</v>
       </c>
       <c r="G17" s="1">
-        <v>216</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -925,19 +928,19 @@
         <v>8</v>
       </c>
       <c r="C18" s="3">
-        <v>34543.62</v>
+        <v>11514.54</v>
       </c>
       <c r="D18" s="3">
-        <v>168122.28</v>
+        <v>56040.76</v>
       </c>
       <c r="E18" s="3">
         <v>2444.44</v>
       </c>
       <c r="F18" s="3">
-        <v>2.852767969898418</v>
+        <v>1.418258787877028</v>
       </c>
       <c r="G18" s="1">
-        <v>117</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -948,19 +951,19 @@
         <v>7</v>
       </c>
       <c r="C19" s="3">
-        <v>97517.75999999999</v>
+        <v>32505.92</v>
       </c>
       <c r="D19" s="3">
-        <v>450581.97</v>
+        <v>150193.99</v>
       </c>
       <c r="E19" s="3">
         <v>3229.17</v>
       </c>
       <c r="F19" s="3">
-        <v>2.079086577095331</v>
+        <v>1.622269401480327</v>
       </c>
       <c r="G19" s="1">
-        <v>162</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -971,19 +974,19 @@
         <v>12</v>
       </c>
       <c r="C20" s="3">
-        <v>175218.57</v>
+        <v>58406.19</v>
       </c>
       <c r="D20" s="3">
-        <v>776805.1800000001</v>
+        <v>258935.06</v>
       </c>
       <c r="E20" s="3">
         <v>3666.67</v>
       </c>
       <c r="F20" s="3">
-        <v>2.645684797388774</v>
+        <v>1.806412673934507</v>
       </c>
       <c r="G20" s="1">
-        <v>198</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -994,19 +997,88 @@
         <v>13</v>
       </c>
       <c r="C21" s="3">
-        <v>52391.34</v>
+        <v>17463.78</v>
       </c>
       <c r="D21" s="3">
-        <v>242262.36</v>
+        <v>80754.12</v>
       </c>
       <c r="E21" s="3">
         <v>2291.67</v>
       </c>
       <c r="F21" s="3">
-        <v>1.810941041535916</v>
+        <v>1.537361423885984</v>
       </c>
       <c r="G21" s="1">
-        <v>144</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="1">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="3">
+        <v>39162.64</v>
+      </c>
+      <c r="D22" s="3">
+        <v>229155.65</v>
+      </c>
+      <c r="E22" s="3">
+        <v>20000</v>
+      </c>
+      <c r="F22" s="3">
+        <v>1.308383284592937</v>
+      </c>
+      <c r="G22" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="1">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="3">
+        <v>140363.06</v>
+      </c>
+      <c r="D23" s="3">
+        <v>710773.53</v>
+      </c>
+      <c r="E23" s="3">
+        <v>31944.44</v>
+      </c>
+      <c r="F23" s="3">
+        <v>1.537361423885984</v>
+      </c>
+      <c r="G23" s="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="1">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="3">
+        <v>71825.78</v>
+      </c>
+      <c r="D24" s="3">
+        <v>377795.57</v>
+      </c>
+      <c r="E24" s="3">
+        <v>43888.89</v>
+      </c>
+      <c r="F24" s="3">
+        <v>1.207020068576251</v>
+      </c>
+      <c r="G24" s="1">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1019,7 +1091,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.5703125" bestFit="1" customWidth="1"/>
@@ -1030,16 +1102,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1050,10 +1122,10 @@
         <v>9</v>
       </c>
       <c r="C2" s="3">
-        <v>17690.01</v>
+        <v>5749.03</v>
       </c>
       <c r="D2" s="3">
-        <v>106425.98</v>
+        <v>34585.24</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1064,10 +1136,10 @@
         <v>11</v>
       </c>
       <c r="C3" s="3">
-        <v>9010.530000000001</v>
+        <v>3003.51</v>
       </c>
       <c r="D3" s="3">
-        <v>53441.79</v>
+        <v>17813.93</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1078,10 +1150,10 @@
         <v>7</v>
       </c>
       <c r="C4" s="3">
-        <v>68652.33</v>
+        <v>22884.11</v>
       </c>
       <c r="D4" s="3">
-        <v>419387.07</v>
+        <v>139795.69</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1089,13 +1161,13 @@
         <v>2009</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C5" s="3">
-        <v>5479.98</v>
+        <v>20639.78</v>
       </c>
       <c r="D5" s="3">
-        <v>33223.44</v>
+        <v>126820.42</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1103,27 +1175,27 @@
         <v>2009</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C6" s="3">
-        <v>9743.6</v>
+        <v>1826.66</v>
       </c>
       <c r="D6" s="3">
-        <v>58214.22</v>
+        <v>11074.48</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C7" s="3">
-        <v>51367.67</v>
+        <v>3054.24</v>
       </c>
       <c r="D7" s="3">
-        <v>283504.48</v>
+        <v>18247.9</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1131,13 +1203,13 @@
         <v>2010</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C8" s="3">
-        <v>6575.94</v>
+        <v>16599.95</v>
       </c>
       <c r="D8" s="3">
-        <v>35803.86</v>
+        <v>91633.2</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1145,13 +1217,13 @@
         <v>2010</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C9" s="3">
-        <v>39105.36</v>
+        <v>2191.98</v>
       </c>
       <c r="D9" s="3">
-        <v>218454.78</v>
+        <v>11934.62</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1159,13 +1231,13 @@
         <v>2010</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3">
-        <v>145436.61</v>
+        <v>13035.12</v>
       </c>
       <c r="D10" s="3">
-        <v>807095.1</v>
+        <v>72818.25999999999</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1173,13 +1245,13 @@
         <v>2010</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C11" s="3">
-        <v>25233.45</v>
+        <v>48478.87</v>
       </c>
       <c r="D11" s="3">
-        <v>138693.48</v>
+        <v>269031.7</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1187,13 +1259,13 @@
         <v>2010</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" s="3">
-        <v>64256.5</v>
+        <v>8411.15</v>
       </c>
       <c r="D12" s="3">
-        <v>353759.17</v>
+        <v>46231.16</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1201,13 +1273,13 @@
         <v>2010</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C13" s="3">
-        <v>19002.54</v>
+        <v>20747.54</v>
       </c>
       <c r="D13" s="3">
-        <v>104809.47</v>
+        <v>114201.81</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -1215,41 +1287,41 @@
         <v>2010</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C14" s="3">
-        <v>75325.53</v>
+        <v>108879.44</v>
       </c>
       <c r="D14" s="3">
-        <v>414557.31</v>
+        <v>601834.23</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C15" s="3">
-        <v>64155.9</v>
+        <v>6334.18</v>
       </c>
       <c r="D15" s="3">
-        <v>321018.2</v>
+        <v>34936.49</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="1">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C16" s="3">
-        <v>8027.79</v>
+        <v>24563.93</v>
       </c>
       <c r="D16" s="3">
-        <v>40293.66</v>
+        <v>135150.77</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1257,13 +1329,13 @@
         <v>2011</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C17" s="3">
-        <v>21027.09</v>
+        <v>20587.04</v>
       </c>
       <c r="D17" s="3">
-        <v>105845.13</v>
+        <v>103013.78</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -1271,13 +1343,13 @@
         <v>2011</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C18" s="3">
-        <v>142821.12</v>
+        <v>2675.93</v>
       </c>
       <c r="D18" s="3">
-        <v>715602.9300000001</v>
+        <v>13431.22</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -1285,13 +1357,13 @@
         <v>2011</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C19" s="3">
-        <v>45747.9</v>
+        <v>7009.03</v>
       </c>
       <c r="D19" s="3">
-        <v>229116.63</v>
+        <v>35281.71</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -1299,13 +1371,13 @@
         <v>2011</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C20" s="3">
-        <v>111736.71</v>
+        <v>47607.04</v>
       </c>
       <c r="D20" s="3">
-        <v>559013.67</v>
+        <v>238534.31</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -1313,13 +1385,13 @@
         <v>2011</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C21" s="3">
-        <v>21140.82</v>
+        <v>15249.3</v>
       </c>
       <c r="D21" s="3">
-        <v>106238.88</v>
+        <v>76372.21000000001</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -1327,55 +1399,55 @@
         <v>2011</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C22" s="3">
-        <v>86186.3</v>
+        <v>36553.19</v>
       </c>
       <c r="D22" s="3">
-        <v>431429.2</v>
+        <v>182873.91</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="1">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C23" s="3">
-        <v>50301.92</v>
+        <v>82524.02</v>
       </c>
       <c r="D23" s="3">
-        <v>226324.72</v>
+        <v>415649.92</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="1">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C24" s="3">
-        <v>3928.5</v>
+        <v>7046.94</v>
       </c>
       <c r="D24" s="3">
-        <v>17791.74</v>
+        <v>35412.96</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="1">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C25" s="3">
-        <v>7290</v>
+        <v>28297.94</v>
       </c>
       <c r="D25" s="3">
-        <v>33177.42</v>
+        <v>141651.92</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -1383,13 +1455,13 @@
         <v>2012</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C26" s="3">
-        <v>96545.64</v>
+        <v>16108.16</v>
       </c>
       <c r="D26" s="3">
-        <v>435085.35</v>
+        <v>72477.42</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -1397,13 +1469,13 @@
         <v>2012</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C27" s="3">
-        <v>33733.68</v>
+        <v>1309.5</v>
       </c>
       <c r="D27" s="3">
-        <v>151850.31</v>
+        <v>5930.58</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1411,13 +1483,13 @@
         <v>2012</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C28" s="3">
-        <v>92557.09</v>
+        <v>2430</v>
       </c>
       <c r="D28" s="3">
-        <v>416124.59</v>
+        <v>11059.14</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -1425,13 +1497,13 @@
         <v>2012</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C29" s="3">
-        <v>9728.16</v>
+        <v>32181.88</v>
       </c>
       <c r="D29" s="3">
-        <v>43969.11</v>
+        <v>145028.45</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -1439,69 +1511,69 @@
         <v>2012</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C30" s="3">
-        <v>68338.89999999999</v>
+        <v>11244.56</v>
       </c>
       <c r="D30" s="3">
-        <v>307364.6</v>
+        <v>50616.77</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="1">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C31" s="3">
-        <v>35056.01</v>
+        <v>30263.85</v>
       </c>
       <c r="D31" s="3">
-        <v>141815.52</v>
+        <v>136063.21</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="1">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C32" s="3">
-        <v>427.05</v>
+        <v>29337.08</v>
       </c>
       <c r="D32" s="3">
-        <v>1785.66</v>
+        <v>132578.45</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C33" s="3">
-        <v>81</v>
+        <v>3242.72</v>
       </c>
       <c r="D33" s="3">
-        <v>342.75</v>
+        <v>14656.37</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="1">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C34" s="3">
-        <v>50113.8</v>
+        <v>22464.98</v>
       </c>
       <c r="D34" s="3">
-        <v>203580.12</v>
+        <v>101038.3</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -1509,13 +1581,13 @@
         <v>2013</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C35" s="3">
-        <v>21719.34</v>
+        <v>11186.95</v>
       </c>
       <c r="D35" s="3">
-        <v>87955.38</v>
+        <v>45257.68</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -1523,13 +1595,13 @@
         <v>2013</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C36" s="3">
-        <v>72517.89</v>
+        <v>142.35</v>
       </c>
       <c r="D36" s="3">
-        <v>292951.34</v>
+        <v>595.22</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -1537,13 +1609,13 @@
         <v>2013</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C37" s="3">
-        <v>2945.58</v>
+        <v>27</v>
       </c>
       <c r="D37" s="3">
-        <v>12100.5</v>
+        <v>114.25</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -1551,223 +1623,293 @@
         <v>2013</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C38" s="3">
-        <v>50491.48</v>
+        <v>16704.6</v>
       </c>
       <c r="D38" s="3">
-        <v>204110.57</v>
+        <v>67860.03999999999</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="1">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C39" s="3">
-        <v>21693.03</v>
+        <v>7239.78</v>
       </c>
       <c r="D39" s="3">
-        <v>78845.64</v>
+        <v>29318.46</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="1">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C40" s="3">
-        <v>11609.55</v>
+        <v>23688.79</v>
       </c>
       <c r="D40" s="3">
-        <v>42840.93</v>
+        <v>95696.89999999999</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="1">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C41" s="3">
-        <v>9705.42</v>
+        <v>9971.16</v>
       </c>
       <c r="D41" s="3">
-        <v>35510.82</v>
+        <v>40841.73</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="1">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C42" s="3">
-        <v>52479.12</v>
+        <v>981.86</v>
       </c>
       <c r="D42" s="3">
-        <v>190567.75</v>
+        <v>4033.5</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="1">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C43" s="3">
-        <v>32644.03</v>
+        <v>16632.02</v>
       </c>
       <c r="D43" s="3">
-        <v>118713.75</v>
+        <v>67232.89</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="1">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C44" s="3">
-        <v>11342.6</v>
+        <v>6893.43</v>
       </c>
       <c r="D44" s="3">
-        <v>37162.87</v>
+        <v>25055</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="1">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C45" s="3">
-        <v>399.66</v>
+        <v>3869.85</v>
       </c>
       <c r="D45" s="3">
-        <v>1355.79</v>
+        <v>14280.31</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="1">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C46" s="3">
-        <v>1399.68</v>
+        <v>3235.14</v>
       </c>
       <c r="D46" s="3">
-        <v>4678.47</v>
+        <v>11836.94</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="1">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C47" s="3">
-        <v>32440.15</v>
+        <v>17113.8</v>
       </c>
       <c r="D47" s="3">
-        <v>106012.99</v>
+        <v>62146.75</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="1">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C48" s="3">
-        <v>16623.54</v>
+        <v>10799.05</v>
       </c>
       <c r="D48" s="3">
-        <v>54393.64</v>
+        <v>39269.67</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="1">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C49" s="3">
-        <v>1852.42</v>
+        <v>3604.08</v>
       </c>
       <c r="D49" s="3">
-        <v>5581.21</v>
+        <v>11808.39</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="1">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C50" s="3">
-        <v>14641.42</v>
+        <v>133.22</v>
       </c>
       <c r="D50" s="3">
-        <v>43051.32</v>
+        <v>451.93</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="1">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C51" s="3">
-        <v>4583.82</v>
+        <v>466.56</v>
       </c>
       <c r="D51" s="3">
-        <v>13678.98</v>
+        <v>1559.49</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="1">
-        <v>2017</v>
+        <v>2015</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C52" s="3">
-        <v>5323.52</v>
+        <v>10538.73</v>
       </c>
       <c r="D52" s="3">
-        <v>14152.89</v>
+        <v>34441.99</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="1">
+        <v>2015</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" s="3">
+        <v>5538.76</v>
+      </c>
+      <c r="D53" s="3">
+        <v>18122.98</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="1">
+        <v>2016</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="3">
+        <v>588.62</v>
+      </c>
+      <c r="D54" s="3">
+        <v>1773.47</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" s="1">
+        <v>2016</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C55" s="3">
+        <v>4710.48</v>
+      </c>
+      <c r="D55" s="3">
+        <v>13851.56</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="1">
+        <v>2016</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" s="3">
+        <v>1527.94</v>
+      </c>
+      <c r="D56" s="3">
+        <v>4559.66</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="1">
+        <v>2017</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C57" s="3">
+        <v>1709.12</v>
+      </c>
+      <c r="D57" s="3">
+        <v>4543.81</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="1">
         <v>2018</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B58" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C53" s="3">
-        <v>59.15</v>
-      </c>
-      <c r="D53" s="3">
-        <v>146.2</v>
+      <c r="C58" s="3">
+        <v>18.99</v>
+      </c>
+      <c r="D58" s="3">
+        <v>46.94</v>
       </c>
     </row>
   </sheetData>
@@ -1780,7 +1922,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="53.28515625" bestFit="1" customWidth="1"/>
@@ -1794,125 +1936,139 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
         <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B2" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C2" s="3">
-        <v>515578.71</v>
+        <v>251351.48</v>
       </c>
       <c r="D2" s="3">
-        <v>2624947.29</v>
+        <v>1317724.75</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3">
-        <v>446011.55</v>
+        <v>171859.57</v>
       </c>
       <c r="D3" s="3">
-        <v>1975779.92</v>
+        <v>874982.4300000001</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
       <c r="C4" s="3">
-        <v>343937.2</v>
+        <v>145344.49</v>
       </c>
       <c r="D4" s="3">
-        <v>1602462.27</v>
+        <v>643866.88</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" s="3">
-        <v>253459.56</v>
+        <v>112878.86</v>
       </c>
       <c r="D5" s="3">
-        <v>1200678.62</v>
+        <v>525274.09</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B6" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" s="3">
-        <v>137539.47</v>
+        <v>81317.25999999999</v>
       </c>
       <c r="D6" s="3">
-        <v>647805.09</v>
+        <v>385604.18</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1">
         <v>2</v>
       </c>
       <c r="C7" s="3">
-        <v>76513.98</v>
+        <v>45846.49</v>
       </c>
       <c r="D7" s="3">
-        <v>411261.87</v>
+        <v>215935.03</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B8" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C8" s="3">
-        <v>58297.08</v>
+        <v>25504.66</v>
       </c>
       <c r="D8" s="3">
-        <v>300341.4</v>
+        <v>137087.29</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1">
+        <v>3</v>
+      </c>
+      <c r="C9" s="3">
+        <v>19432.36</v>
+      </c>
+      <c r="D9" s="3">
+        <v>100113.8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B10" s="1">
         <v>1</v>
       </c>
-      <c r="C9" s="3">
-        <v>18959.28</v>
-      </c>
-      <c r="D9" s="3">
-        <v>95674.92</v>
+      <c r="C10" s="3">
+        <v>6319.76</v>
+      </c>
+      <c r="D10" s="3">
+        <v>31891.64</v>
       </c>
     </row>
   </sheetData>
@@ -1936,13 +2092,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
         <v>6</v>
@@ -1953,13 +2109,13 @@
         <v>2009</v>
       </c>
       <c r="B2" s="3">
-        <v>110576.45</v>
+        <v>57157.33</v>
       </c>
       <c r="C2" s="3">
-        <v>670692.5</v>
+        <v>348337.66</v>
       </c>
       <c r="D2" s="1">
-        <v>141</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1967,13 +2123,13 @@
         <v>2010</v>
       </c>
       <c r="B3" s="3">
-        <v>426303.6</v>
+        <v>249242.16</v>
       </c>
       <c r="C3" s="3">
-        <v>2356677.65</v>
+        <v>1377772.24</v>
       </c>
       <c r="D3" s="1">
-        <v>540</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1981,13 +2137,13 @@
         <v>2011</v>
       </c>
       <c r="B4" s="3">
-        <v>500843.63</v>
+        <v>247550.43</v>
       </c>
       <c r="C4" s="3">
-        <v>2508558.3</v>
+        <v>1242221.94</v>
       </c>
       <c r="D4" s="1">
-        <v>711</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1995,13 +2151,13 @@
         <v>2012</v>
       </c>
       <c r="B5" s="3">
-        <v>362423.89</v>
+        <v>148582.73</v>
       </c>
       <c r="C5" s="3">
-        <v>1631687.84</v>
+        <v>669448.6899999999</v>
       </c>
       <c r="D5" s="1">
-        <v>627</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2009,13 +2165,13 @@
         <v>2013</v>
       </c>
       <c r="B6" s="3">
-        <v>233352.15</v>
+        <v>86574.50999999999</v>
       </c>
       <c r="C6" s="3">
-        <v>944641.84</v>
+        <v>350950.67</v>
       </c>
       <c r="D6" s="1">
-        <v>543</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2023,13 +2179,13 @@
         <v>2014</v>
       </c>
       <c r="B7" s="3">
-        <v>128131.15</v>
+        <v>41911.27</v>
       </c>
       <c r="C7" s="3">
-        <v>466478.89</v>
+        <v>152588.67</v>
       </c>
       <c r="D7" s="1">
-        <v>375</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2037,13 +2193,13 @@
         <v>2015</v>
       </c>
       <c r="B8" s="3">
-        <v>62205.63</v>
+        <v>20281.35</v>
       </c>
       <c r="C8" s="3">
-        <v>203603.76</v>
+        <v>66384.78</v>
       </c>
       <c r="D8" s="1">
-        <v>219</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2051,13 +2207,13 @@
         <v>2016</v>
       </c>
       <c r="B9" s="3">
-        <v>21077.66</v>
+        <v>6827.04</v>
       </c>
       <c r="C9" s="3">
-        <v>62311.51</v>
+        <v>20184.69</v>
       </c>
       <c r="D9" s="1">
-        <v>117</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2065,13 +2221,13 @@
         <v>2017</v>
       </c>
       <c r="B10" s="3">
-        <v>5323.52</v>
+        <v>1709.12</v>
       </c>
       <c r="C10" s="3">
-        <v>14152.89</v>
+        <v>4543.81</v>
       </c>
       <c r="D10" s="1">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2079,13 +2235,13 @@
         <v>2018</v>
       </c>
       <c r="B11" s="3">
-        <v>59.15</v>
+        <v>18.99</v>
       </c>
       <c r="C11" s="3">
-        <v>146.2</v>
+        <v>46.94</v>
       </c>
       <c r="D11" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2107,50 +2263,50 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3">
-        <v>1850296.83</v>
+        <v>859854.9300000001</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="3">
-        <v>8858951.380000001</v>
+        <v>4232480.09</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="3">
         <v>23</v>
-      </c>
-      <c r="B4" s="3">
-        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" s="3">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" s="3">
-        <v>3312</v>
+        <v>1203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>